<commit_message>
Update INFO.xlsx with latest data
</commit_message>
<xml_diff>
--- a/INFO.xlsx
+++ b/INFO.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ezzat.rajab.AD\claude-workspace\VGR Alla enheter\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ezzat.rajab.AD\claude-workspace\VGR Alla enheter\Dashboard\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A67F657-C1DC-4C3E-BAFC-27EBF1FC2DCB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8449C5C3-3D19-4BCE-99CF-858B65102402}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{C7EECDDD-B360-4ED3-93ED-44C91AA1DB71}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C7EECDDD-B360-4ED3-93ED-44C91AA1DB71}"/>
   </bookViews>
   <sheets>
     <sheet name="INFO" sheetId="1" r:id="rId1"/>
@@ -425,7 +425,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0.##;\-#,##0.##"/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -434,11 +434,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <name val="Aptos Narrow"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <name val="Aptos Narrow"/>
     </font>
@@ -570,7 +565,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -584,34 +579,32 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="37" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -6853,37 +6846,37 @@
       <c r="A78" t="s">
         <v>9</v>
       </c>
-      <c r="B78" s="10">
+      <c r="B78" s="9">
         <v>3917066.4</v>
       </c>
-      <c r="C78" s="10">
+      <c r="C78" s="9">
         <v>3872097.84</v>
       </c>
-      <c r="D78" s="10">
+      <c r="D78" s="9">
         <v>3825168.38</v>
       </c>
-      <c r="E78" s="10">
+      <c r="E78" s="9">
         <v>3851675.29</v>
       </c>
-      <c r="F78" s="10">
+      <c r="F78" s="9">
         <v>3843038.29</v>
       </c>
-      <c r="G78" s="10">
+      <c r="G78" s="9">
         <v>3912562.48</v>
       </c>
-      <c r="H78" s="10">
+      <c r="H78" s="9">
         <v>3839706.1</v>
       </c>
-      <c r="I78" s="10">
+      <c r="I78" s="9">
         <v>3856861.96</v>
       </c>
-      <c r="J78" s="10">
+      <c r="J78" s="9">
         <v>3853885.38</v>
       </c>
-      <c r="K78" s="10">
+      <c r="K78" s="9">
         <v>3824597.03</v>
       </c>
-      <c r="L78" s="10">
+      <c r="L78" s="9">
         <v>3945506.72</v>
       </c>
       <c r="N78" s="4" t="s">
@@ -6894,37 +6887,37 @@
       <c r="A79" t="s">
         <v>11</v>
       </c>
-      <c r="B79" s="10">
+      <c r="B79" s="9">
         <v>3368631.08</v>
       </c>
-      <c r="C79" s="10">
+      <c r="C79" s="9">
         <v>3423719.12</v>
       </c>
-      <c r="D79" s="10">
+      <c r="D79" s="9">
         <v>3402807.88</v>
       </c>
-      <c r="E79" s="10">
+      <c r="E79" s="9">
         <v>3422269.07</v>
       </c>
-      <c r="F79" s="10">
+      <c r="F79" s="9">
         <v>3401896.2</v>
       </c>
-      <c r="G79" s="10">
+      <c r="G79" s="9">
         <v>3513213.78</v>
       </c>
-      <c r="H79" s="10">
+      <c r="H79" s="9">
         <v>3626781.46</v>
       </c>
-      <c r="I79" s="10">
+      <c r="I79" s="9">
         <v>3467379.04</v>
       </c>
-      <c r="J79" s="10">
+      <c r="J79" s="9">
         <v>3386149.11</v>
       </c>
-      <c r="K79" s="10">
+      <c r="K79" s="9">
         <v>3389868.87</v>
       </c>
-      <c r="L79" s="10">
+      <c r="L79" s="9">
         <v>3341888.68</v>
       </c>
       <c r="N79" s="4" t="s">
@@ -6935,37 +6928,37 @@
       <c r="A80" t="s">
         <v>13</v>
       </c>
-      <c r="B80" s="10">
+      <c r="B80" s="9">
         <v>3328626.22</v>
       </c>
-      <c r="C80" s="10">
+      <c r="C80" s="9">
         <v>3438837.34</v>
       </c>
-      <c r="D80" s="10">
+      <c r="D80" s="9">
         <v>3267125.04</v>
       </c>
-      <c r="E80" s="10">
+      <c r="E80" s="9">
         <v>3300519.45</v>
       </c>
-      <c r="F80" s="10">
+      <c r="F80" s="9">
         <v>3334236.01</v>
       </c>
-      <c r="G80" s="10">
+      <c r="G80" s="9">
         <v>3373971.45</v>
       </c>
-      <c r="H80" s="10">
+      <c r="H80" s="9">
         <v>3526722.97</v>
       </c>
-      <c r="I80" s="10">
+      <c r="I80" s="9">
         <v>3429226.66</v>
       </c>
-      <c r="J80" s="10">
+      <c r="J80" s="9">
         <v>3362582.38</v>
       </c>
-      <c r="K80" s="10">
+      <c r="K80" s="9">
         <v>3354727.85</v>
       </c>
-      <c r="L80" s="10">
+      <c r="L80" s="9">
         <v>3365258.2</v>
       </c>
       <c r="N80" s="4" t="s">
@@ -6976,37 +6969,37 @@
       <c r="A81" t="s">
         <v>15</v>
       </c>
-      <c r="B81" s="10">
+      <c r="B81" s="9">
         <v>5517132.7300000004</v>
       </c>
-      <c r="C81" s="10">
+      <c r="C81" s="9">
         <v>5616905.0700000003</v>
       </c>
-      <c r="D81" s="10">
+      <c r="D81" s="9">
         <v>5653617.2800000003</v>
       </c>
-      <c r="E81" s="10">
+      <c r="E81" s="9">
         <v>5633210.0499999998</v>
       </c>
-      <c r="F81" s="10">
+      <c r="F81" s="9">
         <v>5632108.71</v>
       </c>
-      <c r="G81" s="10">
+      <c r="G81" s="9">
         <v>5716619.0099999998</v>
       </c>
-      <c r="H81" s="10">
+      <c r="H81" s="9">
         <v>5948038.2800000003</v>
       </c>
-      <c r="I81" s="10">
+      <c r="I81" s="9">
         <v>5729336.7599999998</v>
       </c>
-      <c r="J81" s="10">
+      <c r="J81" s="9">
         <v>5526525.21</v>
       </c>
-      <c r="K81" s="10">
+      <c r="K81" s="9">
         <v>5743804.46</v>
       </c>
-      <c r="L81" s="10">
+      <c r="L81" s="9">
         <v>5598946.3399999999</v>
       </c>
       <c r="N81" s="4" t="s">
@@ -7017,37 +7010,37 @@
       <c r="A82" t="s">
         <v>17</v>
       </c>
-      <c r="B82" s="10">
+      <c r="B82" s="9">
         <v>6368091.9199999999</v>
       </c>
-      <c r="C82" s="10">
+      <c r="C82" s="9">
         <v>6306013.1399999997</v>
       </c>
-      <c r="D82" s="10">
+      <c r="D82" s="9">
         <v>6370581.6100000003</v>
       </c>
-      <c r="E82" s="10">
+      <c r="E82" s="9">
         <v>6110556.7699999996</v>
       </c>
-      <c r="F82" s="10">
+      <c r="F82" s="9">
         <v>6387107.75</v>
       </c>
-      <c r="G82" s="10">
+      <c r="G82" s="9">
         <v>6405372.7699999996</v>
       </c>
-      <c r="H82" s="10">
+      <c r="H82" s="9">
         <v>6455981.7599999998</v>
       </c>
-      <c r="I82" s="10">
+      <c r="I82" s="9">
         <v>6384454.8200000003</v>
       </c>
-      <c r="J82" s="10">
+      <c r="J82" s="9">
         <v>6432663.7199999997</v>
       </c>
-      <c r="K82" s="10">
+      <c r="K82" s="9">
         <v>6415667.3600000003</v>
       </c>
-      <c r="L82" s="10">
+      <c r="L82" s="9">
         <v>6338936.8499999996</v>
       </c>
       <c r="N82" s="4" t="s">
@@ -7545,37 +7538,37 @@
       <c r="A96" t="s">
         <v>4</v>
       </c>
-      <c r="B96" s="11">
+      <c r="B96">
         <v>-1756104</v>
       </c>
-      <c r="C96" s="11">
+      <c r="C96">
         <v>-1702342.63</v>
       </c>
-      <c r="D96" s="11">
+      <c r="D96">
         <v>-1697754.09</v>
       </c>
-      <c r="E96" s="11">
+      <c r="E96">
         <v>-1687007.65</v>
       </c>
-      <c r="F96" s="11">
+      <c r="F96">
         <v>-1757738.58</v>
       </c>
-      <c r="G96" s="11">
+      <c r="G96">
         <v>-1705786.74</v>
       </c>
-      <c r="H96" s="11">
+      <c r="H96">
         <v>-1692749.91</v>
       </c>
-      <c r="I96" s="11">
+      <c r="I96">
         <v>-1692014.62</v>
       </c>
-      <c r="J96" s="11">
+      <c r="J96">
         <v>-1833474.35</v>
       </c>
-      <c r="K96" s="11">
+      <c r="K96">
         <v>-1722429.48</v>
       </c>
-      <c r="L96" s="11">
+      <c r="L96">
         <v>-1657765.21</v>
       </c>
       <c r="N96" s="4">
@@ -7676,37 +7669,37 @@
       <c r="A100" t="s">
         <v>8</v>
       </c>
-      <c r="B100" s="9">
+      <c r="B100">
         <v>-1154261.45</v>
       </c>
-      <c r="C100" s="9">
+      <c r="C100">
         <v>-1224432.6000000001</v>
       </c>
-      <c r="D100" s="9">
+      <c r="D100">
         <v>-1215399.94</v>
       </c>
-      <c r="E100" s="9">
+      <c r="E100">
         <v>-1193523.72</v>
       </c>
-      <c r="F100" s="9">
+      <c r="F100">
         <v>-1221077.6100000001</v>
       </c>
-      <c r="G100" s="9">
+      <c r="G100">
         <v>-1143467.67</v>
       </c>
-      <c r="H100" s="9">
+      <c r="H100">
         <v>-1187306.71</v>
       </c>
-      <c r="I100" s="9">
+      <c r="I100">
         <v>-1047951.26</v>
       </c>
-      <c r="J100" s="9">
+      <c r="J100">
         <v>-1202726.1200000001</v>
       </c>
-      <c r="K100" s="9">
+      <c r="K100">
         <v>-1168189.73</v>
       </c>
-      <c r="L100" s="9">
+      <c r="L100">
         <v>-1147398.06</v>
       </c>
       <c r="N100" s="4">
@@ -7717,37 +7710,37 @@
       <c r="A101" t="s">
         <v>9</v>
       </c>
-      <c r="B101" s="11">
+      <c r="B101">
         <v>-2614378.7599999998</v>
       </c>
-      <c r="C101" s="11">
+      <c r="C101">
         <v>-2580499.02</v>
       </c>
-      <c r="D101" s="11">
+      <c r="D101">
         <v>-2675716.2400000002</v>
       </c>
-      <c r="E101" s="11">
+      <c r="E101">
         <v>-2637024.02</v>
       </c>
-      <c r="F101" s="11">
+      <c r="F101">
         <v>-2461904.2400000002</v>
       </c>
-      <c r="G101" s="11">
+      <c r="G101">
         <v>-2527042.0499999998</v>
       </c>
-      <c r="H101" s="11">
+      <c r="H101">
         <v>-2617623.56</v>
       </c>
-      <c r="I101" s="11">
+      <c r="I101">
         <v>-2511272.2000000002</v>
       </c>
-      <c r="J101" s="11">
+      <c r="J101">
         <v>-2659781.5</v>
       </c>
-      <c r="K101" s="11">
+      <c r="K101">
         <v>-2485715.0299999998</v>
       </c>
-      <c r="L101" s="11">
+      <c r="L101">
         <v>-2498472.9500000002</v>
       </c>
       <c r="N101" s="4" t="s">
@@ -7758,37 +7751,37 @@
       <c r="A102" t="s">
         <v>11</v>
       </c>
-      <c r="B102" s="11">
+      <c r="B102">
         <v>-1832886.8</v>
       </c>
-      <c r="C102" s="11">
+      <c r="C102">
         <v>-1941634.32</v>
       </c>
-      <c r="D102" s="11">
+      <c r="D102">
         <v>-2004262.58</v>
       </c>
-      <c r="E102" s="11">
+      <c r="E102">
         <v>-1972918.02</v>
       </c>
-      <c r="F102" s="11">
+      <c r="F102">
         <v>-1883024.46</v>
       </c>
-      <c r="G102" s="11">
+      <c r="G102">
         <v>-1900076.23</v>
       </c>
-      <c r="H102" s="11">
+      <c r="H102">
         <v>-1854437.54</v>
       </c>
-      <c r="I102" s="11">
+      <c r="I102">
         <v>-1840429.91</v>
       </c>
-      <c r="J102" s="11">
+      <c r="J102">
         <v>-2076954.93</v>
       </c>
-      <c r="K102" s="11">
+      <c r="K102">
         <v>-1965269.53</v>
       </c>
-      <c r="L102" s="11">
+      <c r="L102">
         <v>-2006046.9</v>
       </c>
       <c r="N102" s="4" t="s">
@@ -7799,37 +7792,37 @@
       <c r="A103" t="s">
         <v>13</v>
       </c>
-      <c r="B103" s="11">
+      <c r="B103">
         <v>-2023957.01</v>
       </c>
-      <c r="C103" s="11">
+      <c r="C103">
         <v>-2017403.68</v>
       </c>
-      <c r="D103" s="11">
+      <c r="D103">
         <v>-2022522.66</v>
       </c>
-      <c r="E103" s="11">
+      <c r="E103">
         <v>-1962640.32</v>
       </c>
-      <c r="F103" s="11">
+      <c r="F103">
         <v>-2015558.93</v>
       </c>
-      <c r="G103" s="11">
+      <c r="G103">
         <v>-1797697.03</v>
       </c>
-      <c r="H103" s="11">
+      <c r="H103">
         <v>-1926810.28</v>
       </c>
-      <c r="I103" s="11">
+      <c r="I103">
         <v>-1970650.55</v>
       </c>
-      <c r="J103" s="11">
+      <c r="J103">
         <v>-2157496.4300000002</v>
       </c>
-      <c r="K103" s="11">
+      <c r="K103">
         <v>-2114754.8199999998</v>
       </c>
-      <c r="L103" s="11">
+      <c r="L103">
         <v>-2055192.29</v>
       </c>
       <c r="N103" s="4" t="s">
@@ -7840,37 +7833,37 @@
       <c r="A104" t="s">
         <v>15</v>
       </c>
-      <c r="B104" s="11">
+      <c r="B104">
         <v>-3078140.84</v>
       </c>
-      <c r="C104" s="11">
+      <c r="C104">
         <v>-3072297.19</v>
       </c>
-      <c r="D104" s="11">
+      <c r="D104">
         <v>-3106626.84</v>
       </c>
-      <c r="E104" s="11">
+      <c r="E104">
         <v>-3205483.86</v>
       </c>
-      <c r="F104" s="11">
+      <c r="F104">
         <v>-2898794.87</v>
       </c>
-      <c r="G104" s="11">
+      <c r="G104">
         <v>-3212275.45</v>
       </c>
-      <c r="H104" s="11">
+      <c r="H104">
         <v>-3227147.65</v>
       </c>
-      <c r="I104" s="11">
+      <c r="I104">
         <v>-3201038.9</v>
       </c>
-      <c r="J104" s="11">
+      <c r="J104">
         <v>-3335956.41</v>
       </c>
-      <c r="K104" s="11">
+      <c r="K104">
         <v>-3093227.95</v>
       </c>
-      <c r="L104" s="11">
+      <c r="L104">
         <v>-3099377.12</v>
       </c>
       <c r="N104" s="4" t="s">
@@ -7881,37 +7874,37 @@
       <c r="A105" t="s">
         <v>17</v>
       </c>
-      <c r="B105" s="11">
+      <c r="B105">
         <v>-3792335.97</v>
       </c>
-      <c r="C105" s="11">
+      <c r="C105">
         <v>-3661595.91</v>
       </c>
-      <c r="D105" s="11">
+      <c r="D105">
         <v>-3225469.59</v>
       </c>
-      <c r="E105" s="11">
+      <c r="E105">
         <v>-3308566.79</v>
       </c>
-      <c r="F105" s="11">
+      <c r="F105">
         <v>-3258231.59</v>
       </c>
-      <c r="G105" s="11">
+      <c r="G105">
         <v>-3068124.1</v>
       </c>
-      <c r="H105" s="11">
+      <c r="H105">
         <v>-3426567.39</v>
       </c>
-      <c r="I105" s="11">
+      <c r="I105">
         <v>-3423675.76</v>
       </c>
-      <c r="J105" s="11">
+      <c r="J105">
         <v>-3587871.31</v>
       </c>
-      <c r="K105" s="11">
+      <c r="K105">
         <v>-3424616.15</v>
       </c>
-      <c r="L105" s="11">
+      <c r="L105">
         <v>-3532843.27</v>
       </c>
       <c r="N105" s="4" t="s">
@@ -8570,37 +8563,37 @@
       <c r="A123" t="s">
         <v>8</v>
       </c>
-      <c r="B123" s="9">
+      <c r="B123">
         <v>-695773.51</v>
       </c>
-      <c r="C123" s="9">
+      <c r="C123">
         <v>-699060.62</v>
       </c>
-      <c r="D123" s="9">
+      <c r="D123">
         <v>-709960.39</v>
       </c>
-      <c r="E123" s="9">
+      <c r="E123">
         <v>-689542.83</v>
       </c>
-      <c r="F123" s="9">
+      <c r="F123">
         <v>-740229.09</v>
       </c>
-      <c r="G123" s="9">
+      <c r="G123">
         <v>-737674.71</v>
       </c>
-      <c r="H123" s="9">
+      <c r="H123">
         <v>-731916.08</v>
       </c>
-      <c r="I123" s="9">
+      <c r="I123">
         <v>-578697.38</v>
       </c>
-      <c r="J123" s="9">
+      <c r="J123">
         <v>-635731.9</v>
       </c>
-      <c r="K123" s="9">
+      <c r="K123">
         <v>-480772.65</v>
       </c>
-      <c r="L123" s="9">
+      <c r="L123">
         <v>-473445.75</v>
       </c>
       <c r="N123" s="4">
@@ -8611,37 +8604,37 @@
       <c r="A124" t="s">
         <v>9</v>
       </c>
-      <c r="B124" s="11">
+      <c r="B124">
         <v>-1371028.13</v>
       </c>
-      <c r="C124" s="11">
+      <c r="C124">
         <v>-1198467.29</v>
       </c>
-      <c r="D124" s="11">
+      <c r="D124">
         <v>-1276632.3799999999</v>
       </c>
-      <c r="E124" s="11">
+      <c r="E124">
         <v>-1161414.4099999999</v>
       </c>
-      <c r="F124" s="11">
+      <c r="F124">
         <v>-1332115.81</v>
       </c>
-      <c r="G124" s="11">
+      <c r="G124">
         <v>-1322340.24</v>
       </c>
-      <c r="H124" s="11">
+      <c r="H124">
         <v>-1112736.97</v>
       </c>
-      <c r="I124" s="11">
+      <c r="I124">
         <v>-1266430.46</v>
       </c>
-      <c r="J124" s="11">
+      <c r="J124">
         <v>-1048214.41</v>
       </c>
-      <c r="K124" s="11">
+      <c r="K124">
         <v>-1169120.2</v>
       </c>
-      <c r="L124" s="11">
+      <c r="L124">
         <v>-1152463.99</v>
       </c>
       <c r="N124" s="4" t="s">
@@ -8652,37 +8645,37 @@
       <c r="A125" t="s">
         <v>11</v>
       </c>
-      <c r="B125" s="11">
+      <c r="B125">
         <v>-1189178.77</v>
       </c>
-      <c r="C125" s="11">
+      <c r="C125">
         <v>-1137215.6499999999</v>
       </c>
-      <c r="D125" s="11">
+      <c r="D125">
         <v>-1246614.5</v>
       </c>
-      <c r="E125" s="11">
+      <c r="E125">
         <v>-933859.13</v>
       </c>
-      <c r="F125" s="11">
+      <c r="F125">
         <v>-1268679.94</v>
       </c>
-      <c r="G125" s="11">
+      <c r="G125">
         <v>-1196830.25</v>
       </c>
-      <c r="H125" s="11">
+      <c r="H125">
         <v>-1111525.69</v>
       </c>
-      <c r="I125" s="11">
+      <c r="I125">
         <v>-1112879.32</v>
       </c>
-      <c r="J125" s="11">
+      <c r="J125">
         <v>-1088019.52</v>
       </c>
-      <c r="K125" s="11">
+      <c r="K125">
         <v>-1031336.83</v>
       </c>
-      <c r="L125" s="11">
+      <c r="L125">
         <v>-956269.07</v>
       </c>
       <c r="N125" s="4" t="s">
@@ -8693,37 +8686,37 @@
       <c r="A126" t="s">
         <v>13</v>
       </c>
-      <c r="B126" s="11">
+      <c r="B126">
         <v>-1023712.98</v>
       </c>
-      <c r="C126" s="11">
+      <c r="C126">
         <v>-838278.48</v>
       </c>
-      <c r="D126" s="11">
+      <c r="D126">
         <v>-974620.39</v>
       </c>
-      <c r="E126" s="11">
+      <c r="E126">
         <v>-875002.07</v>
       </c>
-      <c r="F126" s="11">
+      <c r="F126">
         <v>-975686.34</v>
       </c>
-      <c r="G126" s="11">
+      <c r="G126">
         <v>-892530.68</v>
       </c>
-      <c r="H126" s="11">
+      <c r="H126">
         <v>-918979.24</v>
       </c>
-      <c r="I126" s="11">
+      <c r="I126">
         <v>-940290.06</v>
       </c>
-      <c r="J126" s="11">
+      <c r="J126">
         <v>-919162.63</v>
       </c>
-      <c r="K126" s="11">
+      <c r="K126">
         <v>-824495.46</v>
       </c>
-      <c r="L126" s="11">
+      <c r="L126">
         <v>-860125.87</v>
       </c>
       <c r="N126" s="4" t="s">
@@ -8734,37 +8727,37 @@
       <c r="A127" t="s">
         <v>15</v>
       </c>
-      <c r="B127" s="11">
+      <c r="B127">
         <v>-1892600.35</v>
       </c>
-      <c r="C127" s="11">
+      <c r="C127">
         <v>-1823766.57</v>
       </c>
-      <c r="D127" s="11">
+      <c r="D127">
         <v>-1716357.16</v>
       </c>
-      <c r="E127" s="11">
+      <c r="E127">
         <v>-1680433.69</v>
       </c>
-      <c r="F127" s="11">
+      <c r="F127">
         <v>-1888038.53</v>
       </c>
-      <c r="G127" s="11">
+      <c r="G127">
         <v>-1721641.28</v>
       </c>
-      <c r="H127" s="11">
+      <c r="H127">
         <v>-1905771.55</v>
       </c>
-      <c r="I127" s="11">
+      <c r="I127">
         <v>-1633856.17</v>
       </c>
-      <c r="J127" s="11">
+      <c r="J127">
         <v>-1791170.82</v>
       </c>
-      <c r="K127" s="11">
+      <c r="K127">
         <v>-1731930.81</v>
       </c>
-      <c r="L127" s="11">
+      <c r="L127">
         <v>-1687587.32</v>
       </c>
       <c r="N127" s="4" t="s">
@@ -8775,37 +8768,37 @@
       <c r="A128" t="s">
         <v>17</v>
       </c>
-      <c r="B128" s="11">
+      <c r="B128">
         <v>-1710869.94</v>
       </c>
-      <c r="C128" s="11">
+      <c r="C128">
         <v>-1775835.18</v>
       </c>
-      <c r="D128" s="11">
+      <c r="D128">
         <v>-1627291.75</v>
       </c>
-      <c r="E128" s="11">
+      <c r="E128">
         <v>-1369173.97</v>
       </c>
-      <c r="F128" s="11">
+      <c r="F128">
         <v>-1732346.52</v>
       </c>
-      <c r="G128" s="11">
+      <c r="G128">
         <v>-1751299.87</v>
       </c>
-      <c r="H128" s="11">
+      <c r="H128">
         <v>-1769215.79</v>
       </c>
-      <c r="I128" s="11">
+      <c r="I128">
         <v>-1379357.49</v>
       </c>
-      <c r="J128" s="11">
+      <c r="J128">
         <v>-1617462.33</v>
       </c>
-      <c r="K128" s="11">
+      <c r="K128">
         <v>-1445862.11</v>
       </c>
-      <c r="L128" s="11">
+      <c r="L128">
         <v>-1235094.7</v>
       </c>
       <c r="N128" s="4" t="s">
@@ -9555,43 +9548,43 @@
       </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A26" s="17" t="s">
+      <c r="A26" s="15" t="s">
         <v>118</v>
       </c>
-      <c r="B26" s="17">
+      <c r="B26" s="15">
         <v>202504</v>
       </c>
-      <c r="C26" s="17">
+      <c r="C26" s="15">
         <v>202505</v>
       </c>
-      <c r="D26" s="17">
+      <c r="D26" s="15">
         <v>202506</v>
       </c>
-      <c r="E26" s="17">
+      <c r="E26" s="15">
         <v>202507</v>
       </c>
-      <c r="F26" s="17">
+      <c r="F26" s="15">
         <v>202508</v>
       </c>
-      <c r="G26" s="17">
+      <c r="G26" s="15">
         <v>202509</v>
       </c>
-      <c r="H26" s="17">
+      <c r="H26" s="15">
         <v>202510</v>
       </c>
-      <c r="I26" s="17">
+      <c r="I26" s="15">
         <v>202511</v>
       </c>
-      <c r="J26" s="17">
+      <c r="J26" s="15">
         <v>202512</v>
       </c>
-      <c r="K26" s="17">
+      <c r="K26" s="15">
         <v>202601</v>
       </c>
-      <c r="L26" s="17">
+      <c r="L26" s="15">
         <v>202602</v>
       </c>
-      <c r="M26" s="17">
+      <c r="M26" s="15">
         <v>202603</v>
       </c>
     </row>
@@ -10208,51 +10201,51 @@
       </c>
     </row>
     <row r="42" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="B42" s="16">
+      <c r="B42" s="14">
         <f t="shared" ref="B42:M42" si="1">SUM(B27:B41)</f>
         <v>572</v>
       </c>
-      <c r="C42" s="16">
+      <c r="C42" s="14">
         <f t="shared" si="1"/>
         <v>475</v>
       </c>
-      <c r="D42" s="16">
+      <c r="D42" s="14">
         <f>SUM(D27:D41)</f>
         <v>462</v>
       </c>
-      <c r="E42" s="16">
+      <c r="E42" s="14">
         <f t="shared" si="1"/>
         <v>339</v>
       </c>
-      <c r="F42" s="16">
+      <c r="F42" s="14">
         <f t="shared" si="1"/>
         <v>358</v>
       </c>
-      <c r="G42" s="16">
+      <c r="G42" s="14">
         <f t="shared" si="1"/>
         <v>661</v>
       </c>
-      <c r="H42" s="16">
+      <c r="H42" s="14">
         <f t="shared" si="1"/>
         <v>514</v>
       </c>
-      <c r="I42" s="16">
+      <c r="I42" s="14">
         <f t="shared" si="1"/>
         <v>522</v>
       </c>
-      <c r="J42" s="16">
+      <c r="J42" s="14">
         <f t="shared" si="1"/>
         <v>421</v>
       </c>
-      <c r="K42" s="16">
+      <c r="K42" s="14">
         <f t="shared" si="1"/>
         <v>470</v>
       </c>
-      <c r="L42" s="16">
+      <c r="L42" s="14">
         <f t="shared" si="1"/>
         <v>585</v>
       </c>
-      <c r="M42" s="16">
+      <c r="M42" s="14">
         <f t="shared" si="1"/>
         <v>687</v>
       </c>
@@ -11045,39 +11038,39 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="25" customWidth="1"/>
-    <col min="3" max="3" width="15" style="13" customWidth="1"/>
+    <col min="3" max="3" width="15" style="11" customWidth="1"/>
     <col min="4" max="4" width="25" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:4" ht="23.4" x14ac:dyDescent="0.3">
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="16" t="s">
         <v>88</v>
       </c>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
     </row>
     <row r="3" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B3" s="20" t="s">
+      <c r="B3" s="18" t="s">
         <v>89</v>
       </c>
-      <c r="C3" s="19"/>
-      <c r="D3" s="19"/>
+      <c r="C3" s="17"/>
+      <c r="D3" s="17"/>
     </row>
     <row r="5" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B5" s="21" t="s">
+      <c r="B5" s="19" t="s">
         <v>90</v>
       </c>
-      <c r="C5" s="22"/>
-      <c r="D5" s="23"/>
+      <c r="C5" s="20"/>
+      <c r="D5" s="21"/>
     </row>
     <row r="6" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B6" s="12" t="s">
+      <c r="B6" s="10" t="s">
         <v>92</v>
       </c>
-      <c r="C6" s="14" t="s">
+      <c r="C6" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="D6" s="12" t="s">
+      <c r="D6" s="10" t="s">
         <v>93</v>
       </c>
     </row>
@@ -11085,7 +11078,7 @@
       <c r="B7" t="s">
         <v>33</v>
       </c>
-      <c r="C7" s="13">
+      <c r="C7" s="11">
         <v>102</v>
       </c>
       <c r="D7" t="s">
@@ -11096,7 +11089,7 @@
       <c r="B8" t="s">
         <v>35</v>
       </c>
-      <c r="C8" s="13">
+      <c r="C8" s="11">
         <v>601</v>
       </c>
       <c r="D8" t="s">
@@ -11107,7 +11100,7 @@
       <c r="B9" t="s">
         <v>36</v>
       </c>
-      <c r="C9" s="13">
+      <c r="C9" s="11">
         <v>103</v>
       </c>
       <c r="D9" t="s">
@@ -11118,7 +11111,7 @@
       <c r="B10" t="s">
         <v>37</v>
       </c>
-      <c r="C10" s="13">
+      <c r="C10" s="11">
         <v>602</v>
       </c>
       <c r="D10" t="s">
@@ -11129,7 +11122,7 @@
       <c r="B11" t="s">
         <v>38</v>
       </c>
-      <c r="C11" s="13">
+      <c r="C11" s="11">
         <v>104</v>
       </c>
       <c r="D11" t="s">
@@ -11140,7 +11133,7 @@
       <c r="B12" t="s">
         <v>40</v>
       </c>
-      <c r="C12" s="13">
+      <c r="C12" s="11">
         <v>603</v>
       </c>
       <c r="D12" t="s">
@@ -11151,7 +11144,7 @@
       <c r="B13" t="s">
         <v>41</v>
       </c>
-      <c r="C13" s="13">
+      <c r="C13" s="11">
         <v>106</v>
       </c>
       <c r="D13" t="s">
@@ -11162,7 +11155,7 @@
       <c r="B14" t="s">
         <v>43</v>
       </c>
-      <c r="C14" s="13">
+      <c r="C14" s="11">
         <v>107</v>
       </c>
       <c r="D14" t="s">
@@ -11173,7 +11166,7 @@
       <c r="B15" t="s">
         <v>45</v>
       </c>
-      <c r="C15" s="13">
+      <c r="C15" s="11">
         <v>604</v>
       </c>
       <c r="D15" t="s">
@@ -11184,7 +11177,7 @@
       <c r="B16" t="s">
         <v>46</v>
       </c>
-      <c r="C16" s="13">
+      <c r="C16" s="11">
         <v>108</v>
       </c>
       <c r="D16" t="s">
@@ -11195,7 +11188,7 @@
       <c r="B17" t="s">
         <v>48</v>
       </c>
-      <c r="C17" s="13">
+      <c r="C17" s="11">
         <v>605</v>
       </c>
       <c r="D17" t="s">
@@ -11206,7 +11199,7 @@
       <c r="B18" t="s">
         <v>49</v>
       </c>
-      <c r="C18" s="13">
+      <c r="C18" s="11">
         <v>109</v>
       </c>
       <c r="D18" t="s">
@@ -11217,7 +11210,7 @@
       <c r="B19" t="s">
         <v>50</v>
       </c>
-      <c r="C19" s="13">
+      <c r="C19" s="11">
         <v>110</v>
       </c>
       <c r="D19" t="s">
@@ -11228,7 +11221,7 @@
       <c r="B20" t="s">
         <v>52</v>
       </c>
-      <c r="C20" s="13">
+      <c r="C20" s="11">
         <v>111</v>
       </c>
       <c r="D20" t="s">
@@ -11239,7 +11232,7 @@
       <c r="B21" t="s">
         <v>54</v>
       </c>
-      <c r="C21" s="13">
+      <c r="C21" s="11">
         <v>607</v>
       </c>
       <c r="D21" t="s">
@@ -11250,7 +11243,7 @@
       <c r="B22" t="s">
         <v>55</v>
       </c>
-      <c r="C22" s="13">
+      <c r="C22" s="11">
         <v>302</v>
       </c>
       <c r="D22" t="s">
@@ -11261,7 +11254,7 @@
       <c r="B23" t="s">
         <v>57</v>
       </c>
-      <c r="C23" s="13">
+      <c r="C23" s="11">
         <v>660</v>
       </c>
       <c r="D23" t="s">
@@ -11272,7 +11265,7 @@
       <c r="B24" t="s">
         <v>58</v>
       </c>
-      <c r="C24" s="13">
+      <c r="C24" s="11">
         <v>303</v>
       </c>
       <c r="D24" t="s">
@@ -11283,7 +11276,7 @@
       <c r="B25" t="s">
         <v>59</v>
       </c>
-      <c r="C25" s="13">
+      <c r="C25" s="11">
         <v>304</v>
       </c>
       <c r="D25" t="s">
@@ -11294,7 +11287,7 @@
       <c r="B26" t="s">
         <v>60</v>
       </c>
-      <c r="C26" s="15" t="s">
+      <c r="C26" s="13" t="s">
         <v>91</v>
       </c>
       <c r="D26" t="s">
@@ -11305,7 +11298,7 @@
       <c r="B27" t="s">
         <v>61</v>
       </c>
-      <c r="C27" s="13">
+      <c r="C27" s="11">
         <v>715</v>
       </c>
       <c r="D27" t="s">
@@ -11316,7 +11309,7 @@
       <c r="B28" t="s">
         <v>62</v>
       </c>
-      <c r="C28" s="13">
+      <c r="C28" s="11">
         <v>4020</v>
       </c>
       <c r="D28" t="s">
@@ -11327,7 +11320,7 @@
       <c r="B29" t="s">
         <v>64</v>
       </c>
-      <c r="C29" s="13">
+      <c r="C29" s="11">
         <v>4001</v>
       </c>
       <c r="D29" t="s">
@@ -11335,20 +11328,20 @@
       </c>
     </row>
     <row r="31" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B31" s="21" t="s">
+      <c r="B31" s="19" t="s">
         <v>66</v>
       </c>
-      <c r="C31" s="22"/>
-      <c r="D31" s="23"/>
+      <c r="C31" s="20"/>
+      <c r="D31" s="21"/>
     </row>
     <row r="32" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B32" s="12" t="s">
+      <c r="B32" s="10" t="s">
         <v>92</v>
       </c>
-      <c r="C32" s="14" t="s">
+      <c r="C32" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="D32" s="12" t="s">
+      <c r="D32" s="10" t="s">
         <v>93</v>
       </c>
     </row>
@@ -11356,7 +11349,7 @@
       <c r="B33" t="s">
         <v>67</v>
       </c>
-      <c r="C33" s="15" t="s">
+      <c r="C33" s="13" t="s">
         <v>10</v>
       </c>
       <c r="D33" t="s">
@@ -11367,7 +11360,7 @@
       <c r="B34" t="s">
         <v>69</v>
       </c>
-      <c r="C34" s="13">
+      <c r="C34" s="11">
         <v>703</v>
       </c>
       <c r="D34" t="s">
@@ -11378,7 +11371,7 @@
       <c r="B35" t="s">
         <v>70</v>
       </c>
-      <c r="C35" s="15" t="s">
+      <c r="C35" s="13" t="s">
         <v>14</v>
       </c>
       <c r="D35" t="s">
@@ -11389,7 +11382,7 @@
       <c r="B36" t="s">
         <v>72</v>
       </c>
-      <c r="C36" s="13">
+      <c r="C36" s="11">
         <v>705</v>
       </c>
       <c r="D36" t="s">
@@ -11400,7 +11393,7 @@
       <c r="B37" t="s">
         <v>73</v>
       </c>
-      <c r="C37" s="15" t="s">
+      <c r="C37" s="13" t="s">
         <v>12</v>
       </c>
       <c r="D37" t="s">
@@ -11411,7 +11404,7 @@
       <c r="B38" t="s">
         <v>75</v>
       </c>
-      <c r="C38" s="13">
+      <c r="C38" s="11">
         <v>706</v>
       </c>
       <c r="D38" t="s">
@@ -11422,7 +11415,7 @@
       <c r="B39" t="s">
         <v>76</v>
       </c>
-      <c r="C39" s="15" t="s">
+      <c r="C39" s="13" t="s">
         <v>16</v>
       </c>
       <c r="D39" t="s">
@@ -11433,7 +11426,7 @@
       <c r="B40" t="s">
         <v>78</v>
       </c>
-      <c r="C40" s="13">
+      <c r="C40" s="11">
         <v>708</v>
       </c>
       <c r="D40" t="s">
@@ -11444,7 +11437,7 @@
       <c r="B41" t="s">
         <v>79</v>
       </c>
-      <c r="C41" s="15" t="s">
+      <c r="C41" s="13" t="s">
         <v>18</v>
       </c>
       <c r="D41" t="s">
@@ -11455,7 +11448,7 @@
       <c r="B42" t="s">
         <v>81</v>
       </c>
-      <c r="C42" s="13">
+      <c r="C42" s="11">
         <v>714</v>
       </c>
       <c r="D42" t="s">
@@ -11466,7 +11459,7 @@
       <c r="B43" t="s">
         <v>82</v>
       </c>
-      <c r="C43" s="13">
+      <c r="C43" s="11">
         <v>305</v>
       </c>
       <c r="D43" t="s">
@@ -11477,7 +11470,7 @@
       <c r="B44" t="s">
         <v>84</v>
       </c>
-      <c r="C44" s="13">
+      <c r="C44" s="11">
         <v>670</v>
       </c>
       <c r="D44" t="s">
@@ -11488,7 +11481,7 @@
       <c r="B45" t="s">
         <v>85</v>
       </c>
-      <c r="C45" s="13">
+      <c r="C45" s="11">
         <v>650</v>
       </c>
       <c r="D45" t="s">
@@ -11499,7 +11492,7 @@
       <c r="B46" t="s">
         <v>86</v>
       </c>
-      <c r="C46" s="13">
+      <c r="C46" s="11">
         <v>713</v>
       </c>
       <c r="D46" t="s">
@@ -11507,11 +11500,11 @@
       </c>
     </row>
     <row r="48" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B48" s="24" t="s">
+      <c r="B48" s="22" t="s">
         <v>87</v>
       </c>
-      <c r="C48" s="19"/>
-      <c r="D48" s="19"/>
+      <c r="C48" s="17"/>
+      <c r="D48" s="17"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>